<commit_message>
DPMDP v1.0 status updated for July 27
</commit_message>
<xml_diff>
--- a/testing/DPMDP_Status.xlsx
+++ b/testing/DPMDP_Status.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\KarthikeyanV\DPMDP-excel-status\testing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\KarthikeyanV\Node-Workspace\DPMDP-excel-status\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74C5254D-50B3-4F7E-9EF9-5E88043CD412}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05C2D21C-3EEC-460A-92A2-852DB9B31196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CBC9CF17-1400-437B-9968-9867189262AD}"/>
   </bookViews>
   <sheets>
-    <sheet name="0724" sheetId="4" r:id="rId1"/>
-    <sheet name="0722" sheetId="3" r:id="rId2"/>
-    <sheet name="0710" sheetId="1" r:id="rId3"/>
-    <sheet name="0626" sheetId="2" r:id="rId4"/>
+    <sheet name="0727" sheetId="5" r:id="rId1"/>
+    <sheet name="0724" sheetId="4" r:id="rId2"/>
+    <sheet name="0722" sheetId="3" r:id="rId3"/>
+    <sheet name="0710" sheetId="1" r:id="rId4"/>
+    <sheet name="0626" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="43">
   <si>
     <t>p1StreamPmData</t>
   </si>
@@ -138,6 +139,39 @@
   </si>
   <si>
     <t>DPMDP Implementation and Integration Status</t>
+  </si>
+  <si>
+    <t>Spalte1</t>
+  </si>
+  <si>
+    <t>Integrated2</t>
+  </si>
+  <si>
+    <t>Tested3</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>In progress</t>
+  </si>
+  <si>
+    <t>Query by Thorsten: Check in testing if MWDI ES can be replicated by further consuming applications (e.g. MDOI proxy, etc.)</t>
+  </si>
+  <si>
+    <t>Schema validation failed : Actual equipement / physical propreties / temperature should not be required --&gt; FIXED</t>
+  </si>
+  <si>
+    <t>no HPD is returned :Utilzation could not be calculated because of missing agregation group</t>
+  </si>
+  <si>
+    <t>Utilzation could not be calculated because of missing agregation group --&gt; FIX included in DPMDP v1.1</t>
+  </si>
+  <si>
+    <t>Format according tho the schemas</t>
+  </si>
+  <si>
+    <t>batchtimestamp : need to get it from resultCC instead of having time of execution --&gt; FIXED</t>
   </si>
 </sst>
 </file>
@@ -170,7 +204,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -183,8 +217,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="21">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -466,11 +506,66 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -500,11 +595,230 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="11">
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF8ED973"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -515,6 +829,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{85936A10-966C-4FA6-84A3-61A31CE23B03}" name="Tabelle13" displayName="Tabelle13" ref="B5:I32" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9" tableBorderDxfId="8">
+  <autoFilter ref="B5:I32" xr:uid="{85936A10-966C-4FA6-84A3-61A31CE23B03}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{5159E12B-A3C0-40F8-BFC3-7DE639C706A2}" name="Spalte1" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{156B8EF1-C593-4083-9D11-36A3E3BEFA80}" name="Implemented" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{30ECADEA-BEA2-4D7D-98BF-3AA5318DDFC6}" name="Tested" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{59DF8195-8A9A-4FB6-8E9D-791D6C40E051}" name="Integrated" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{CAE0A22C-AFDD-4F74-B92A-9164CA85D3AC}" name="Integrated2" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{2552BEAB-5428-47C6-954A-7798C3BC819B}" name="Tested3" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{728D01E3-B53C-4D68-AE4C-8716D69109E3}" name="NPM" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{6C64D771-338B-4439-A9FD-43A37BFE4F34}" name="Remarks" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -833,6 +1164,406 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3E12C11-8B88-45B7-BD25-4E819046FF08}">
+  <dimension ref="B2:I32"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.88671875" customWidth="1"/>
+    <col min="2" max="2" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.88671875" customWidth="1"/>
+    <col min="4" max="7" width="13.5546875" customWidth="1"/>
+    <col min="9" max="9" width="111.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B2" s="18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" s="1" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B6" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="25"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="7"/>
+      <c r="H6" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="32"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B7" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" s="19"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="32"/>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B8" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="19"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="32"/>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B9" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" s="19"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="32"/>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B10" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="19"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="32"/>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B11" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="19"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" s="33"/>
+      <c r="I11" s="34" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B12" s="23" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="19"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="32"/>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B13" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="19"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="33"/>
+      <c r="I13" s="32"/>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B14" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="19"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="33"/>
+      <c r="I14" s="32"/>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B15" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="19"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="32"/>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B16" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="19"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="32" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B17" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="19"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="33"/>
+      <c r="I17" s="32"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B18" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="19"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="20"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="32"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B19" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="19"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="33"/>
+      <c r="I19" s="32"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B20" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="19"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="33"/>
+      <c r="I20" s="32"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B21" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="19"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="33"/>
+      <c r="I21" s="32"/>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B22" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="19"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="32"/>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B23" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="19"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="35"/>
+      <c r="H23" s="33"/>
+      <c r="I23" s="32" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B24" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="19"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="32"/>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B25" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C25" s="19"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="33"/>
+      <c r="I25" s="32"/>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B26" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="19"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="35"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="32" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B27" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="C27" s="19"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="33"/>
+      <c r="I27" s="32"/>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B28" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="19"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="32" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B29" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" s="19"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="20"/>
+      <c r="H29" s="33"/>
+      <c r="I29" s="32" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B30" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" s="19"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="20"/>
+      <c r="H30" s="33"/>
+      <c r="I30" s="32"/>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B31" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="C31" s="19"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="20"/>
+      <c r="H31" s="33"/>
+      <c r="I31" s="32" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B32" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32" s="27"/>
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H32" s="36"/>
+      <c r="I32" s="32"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2FA5E18-19A2-4DA7-9A95-328DE2FBBD0C}">
   <dimension ref="B2:G32"/>
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1145,7 +1876,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6DC10A0-2F8B-491B-B923-1486860B0A91}">
   <dimension ref="B2:G32"/>
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1458,7 +2189,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{014593E6-C137-4A83-B335-8EC85FCC951C}">
   <dimension ref="B2:G32"/>
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1771,7 +2502,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B872F986-AA11-4310-9F15-06BC0BD7DCB4}">
   <dimension ref="B4:G33"/>
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
DPMDP v1.0 status updated for July 29
</commit_message>
<xml_diff>
--- a/testing/DPMDP_Status.xlsx
+++ b/testing/DPMDP_Status.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\KarthikeyanV\Node-Workspace\DPMDP-excel-status\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05C2D21C-3EEC-460A-92A2-852DB9B31196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA6B8FC6-A4B1-4086-8B43-93D9933107D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CBC9CF17-1400-437B-9968-9867189262AD}"/>
   </bookViews>
   <sheets>
-    <sheet name="0727" sheetId="5" r:id="rId1"/>
-    <sheet name="0724" sheetId="4" r:id="rId2"/>
-    <sheet name="0722" sheetId="3" r:id="rId3"/>
-    <sheet name="0710" sheetId="1" r:id="rId4"/>
-    <sheet name="0626" sheetId="2" r:id="rId5"/>
+    <sheet name="0729" sheetId="6" r:id="rId1"/>
+    <sheet name="0727" sheetId="5" r:id="rId2"/>
+    <sheet name="0724" sheetId="4" r:id="rId3"/>
+    <sheet name="0722" sheetId="3" r:id="rId4"/>
+    <sheet name="0710" sheetId="1" r:id="rId5"/>
+    <sheet name="0626" sheetId="2" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="52">
   <si>
     <t>p1StreamPmData</t>
   </si>
@@ -172,6 +173,67 @@
   </si>
   <si>
     <t>batchtimestamp : need to get it from resultCC instead of having time of execution --&gt; FIXED</t>
+  </si>
+  <si>
+    <t>DPMDP v1.0 Implementation and Integration Status</t>
+  </si>
+  <si>
+    <t>DPMDP v1.1 Implementation and Integration Status</t>
+  </si>
+  <si>
+    <t>Lots</t>
+  </si>
+  <si>
+    <t>P2StreamPmData</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Config json generation </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>completed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Spec analysis </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>in progress</t>
+    </r>
+  </si>
+  <si>
+    <t>P2ProcessDevice</t>
+  </si>
+  <si>
+    <t>P2LoadRawCc</t>
+  </si>
+  <si>
+    <t>P2CreateResultCc</t>
+  </si>
+  <si>
+    <t>P2Storing</t>
   </si>
 </sst>
 </file>
@@ -565,7 +627,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -603,11 +665,21 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="34">
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -640,12 +712,12 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -658,18 +730,16 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -682,18 +752,16 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -706,18 +774,16 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -730,22 +796,32 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
@@ -818,6 +894,426 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF8ED973"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF8ED973"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -832,17 +1328,52 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{85936A10-966C-4FA6-84A3-61A31CE23B03}" name="Tabelle13" displayName="Tabelle13" ref="B5:I32" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9" tableBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3A44319A-9F69-4D9A-9046-8CF13AFDF5EC}" name="Tabelle134" displayName="Tabelle134" ref="B5:I32" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21" tableBorderDxfId="20">
+  <autoFilter ref="B5:I32" xr:uid="{3A44319A-9F69-4D9A-9046-8CF13AFDF5EC}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{58168053-F602-420D-B002-FD9CD5598E51}" name="Spalte1" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{2AC36CD7-C121-4FA9-83EA-0489A955BB3A}" name="Implemented" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{79AD966F-7C25-4A7E-916E-C339B0C4EAF7}" name="Tested" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{762AAEED-7B15-47E8-B3B3-508622706E72}" name="Integrated" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{6F05FA60-3032-40C1-BA87-3A0A10306FA1}" name="Integrated2" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{71F13F73-BD00-4BA9-93AF-0BA612A458FB}" name="Tested3" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{F752B342-AC4E-41AC-844C-BC2883F7EA06}" name="NPM" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{2891536E-8CB5-4D6B-9B8D-96311005FB70}" name="Remarks" dataDxfId="12"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BDD2E654-7D8B-4053-9E09-DC375F5FC6AD}" name="Tabelle1345" displayName="Tabelle1345" ref="B37:J64" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" tableBorderDxfId="9">
+  <autoFilter ref="B37:J64" xr:uid="{BDD2E654-7D8B-4053-9E09-DC375F5FC6AD}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{47586FC5-A2B7-41C5-BD16-5BCE2F84027B}" name="Spalte1" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{7AEE1190-1F6D-446F-B1F3-656DB977BAE2}" name="Implemented" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{18D61296-7463-4D11-A1DE-B39FC2BC3425}" name="Lots" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{79FFD8A3-51F3-48B6-8B47-9F7B013575ED}" name="Tested" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{5D25A49C-0AE1-45D0-B972-D74F10B86940}" name="Integrated" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{9BE68465-7013-4766-8A6B-DB58A21334CF}" name="Integrated2" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{79AC5493-6333-416F-8F72-B099BB3B3C56}" name="Tested3" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{E12BDF81-368B-46E8-8BFA-C2BC19693E94}" name="NPM" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{521D7544-82D4-47BA-87BB-69B1F22D5F3E}" name="Remarks" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{85936A10-966C-4FA6-84A3-61A31CE23B03}" name="Tabelle13" displayName="Tabelle13" ref="B5:I32" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32" tableBorderDxfId="31">
   <autoFilter ref="B5:I32" xr:uid="{85936A10-966C-4FA6-84A3-61A31CE23B03}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{5159E12B-A3C0-40F8-BFC3-7DE639C706A2}" name="Spalte1" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{156B8EF1-C593-4083-9D11-36A3E3BEFA80}" name="Implemented" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{30ECADEA-BEA2-4D7D-98BF-3AA5318DDFC6}" name="Tested" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{59DF8195-8A9A-4FB6-8E9D-791D6C40E051}" name="Integrated" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{CAE0A22C-AFDD-4F74-B92A-9164CA85D3AC}" name="Integrated2" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{2552BEAB-5428-47C6-954A-7798C3BC819B}" name="Tested3" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{728D01E3-B53C-4D68-AE4C-8716D69109E3}" name="NPM" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{6C64D771-338B-4439-A9FD-43A37BFE4F34}" name="Remarks" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{5159E12B-A3C0-40F8-BFC3-7DE639C706A2}" name="Spalte1" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{156B8EF1-C593-4083-9D11-36A3E3BEFA80}" name="Implemented" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{30ECADEA-BEA2-4D7D-98BF-3AA5318DDFC6}" name="Tested" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{59DF8195-8A9A-4FB6-8E9D-791D6C40E051}" name="Integrated" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{CAE0A22C-AFDD-4F74-B92A-9164CA85D3AC}" name="Integrated2" dataDxfId="26"/>
+    <tableColumn id="6" xr3:uid="{2552BEAB-5428-47C6-954A-7798C3BC819B}" name="Tested3" dataDxfId="25"/>
+    <tableColumn id="7" xr3:uid="{728D01E3-B53C-4D68-AE4C-8716D69109E3}" name="NPM" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{6C64D771-338B-4439-A9FD-43A37BFE4F34}" name="Remarks" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1164,6 +1695,771 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54FD33EF-FACE-4D93-A3C0-321F97A1A779}">
+  <dimension ref="B2:J64"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.88671875" customWidth="1"/>
+    <col min="2" max="2" width="44" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="13.5546875" customWidth="1"/>
+    <col min="9" max="9" width="44.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B2" s="18" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" s="1" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B6" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="25"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="7"/>
+      <c r="H6" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="32"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B7" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" s="19"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="32"/>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B8" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="19"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="32"/>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B9" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" s="19"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="32"/>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B10" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="19"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="32"/>
+    </row>
+    <row r="11" spans="2:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B11" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="19"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" s="33"/>
+      <c r="I11" s="37" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B12" s="23" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="19"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="32"/>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B13" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="19"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="33"/>
+      <c r="I13" s="32"/>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B14" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="19"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="33"/>
+      <c r="I14" s="32"/>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B15" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="19"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="32"/>
+    </row>
+    <row r="16" spans="2:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B16" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="19"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="38" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B17" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="19"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="33"/>
+      <c r="I17" s="32"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B18" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="19"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="20"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="32"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B19" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="19"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="33"/>
+      <c r="I19" s="32"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B20" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="19"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="33"/>
+      <c r="I20" s="32"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B21" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="19"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="33"/>
+      <c r="I21" s="32"/>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B22" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="19"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="32"/>
+    </row>
+    <row r="23" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B23" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="19"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="35"/>
+      <c r="H23" s="33"/>
+      <c r="I23" s="38" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B24" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="19"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="32"/>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B25" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C25" s="19"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="33"/>
+      <c r="I25" s="32"/>
+    </row>
+    <row r="26" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B26" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="19"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="35"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="38" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B27" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="C27" s="19"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="33"/>
+      <c r="I27" s="32"/>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B28" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="19"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="32" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B29" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" s="19"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="20"/>
+      <c r="H29" s="33"/>
+      <c r="I29" s="32" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B30" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" s="19"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="20"/>
+      <c r="H30" s="33"/>
+      <c r="I30" s="32"/>
+    </row>
+    <row r="31" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B31" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="C31" s="19"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="20"/>
+      <c r="H31" s="33"/>
+      <c r="I31" s="38" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B32" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32" s="27"/>
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H32" s="36"/>
+      <c r="I32" s="32"/>
+    </row>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B34" s="18" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="36" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B36" s="18"/>
+    </row>
+    <row r="37" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B37" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C37" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="D37" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H37" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="I37" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="J37" s="30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B38" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C38" s="31"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="H38" s="7"/>
+      <c r="I38" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="J38" s="32"/>
+    </row>
+    <row r="39" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B39" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="C39" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="D39" s="40">
+        <v>5</v>
+      </c>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+      <c r="I39" s="33"/>
+      <c r="J39" s="32"/>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B40" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="C40" s="33"/>
+      <c r="D40" s="40">
+        <v>5</v>
+      </c>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="33"/>
+      <c r="J40" s="32"/>
+    </row>
+    <row r="41" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B41" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="C41" s="33"/>
+      <c r="D41" s="40">
+        <v>5</v>
+      </c>
+      <c r="E41" s="3"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+      <c r="I41" s="33"/>
+      <c r="J41" s="32"/>
+    </row>
+    <row r="42" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B42" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="C42" s="33"/>
+      <c r="D42" s="40">
+        <v>5</v>
+      </c>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="33"/>
+      <c r="J42" s="32"/>
+    </row>
+    <row r="43" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B43" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="C43" s="33"/>
+      <c r="D43" s="40">
+        <v>5</v>
+      </c>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="23"/>
+      <c r="I43" s="33"/>
+      <c r="J43" s="32"/>
+    </row>
+    <row r="44" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B44" s="23"/>
+      <c r="C44" s="33"/>
+      <c r="D44" s="12"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+      <c r="I44" s="33"/>
+      <c r="J44" s="32"/>
+    </row>
+    <row r="45" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B45" s="23"/>
+      <c r="C45" s="33"/>
+      <c r="D45" s="12"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="33"/>
+      <c r="J45" s="32"/>
+    </row>
+    <row r="46" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B46" s="23"/>
+      <c r="C46" s="33"/>
+      <c r="D46" s="12"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="33"/>
+      <c r="J46" s="32"/>
+    </row>
+    <row r="47" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B47" s="23"/>
+      <c r="C47" s="33"/>
+      <c r="D47" s="12"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="33"/>
+      <c r="J47" s="32"/>
+    </row>
+    <row r="48" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B48" s="23"/>
+      <c r="C48" s="33"/>
+      <c r="D48" s="12"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="33"/>
+      <c r="J48" s="32"/>
+    </row>
+    <row r="49" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B49" s="23"/>
+      <c r="C49" s="33"/>
+      <c r="D49" s="12"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="33"/>
+      <c r="J49" s="32"/>
+    </row>
+    <row r="50" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B50" s="23"/>
+      <c r="C50" s="33"/>
+      <c r="D50" s="12"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="33"/>
+      <c r="J50" s="32"/>
+    </row>
+    <row r="51" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B51" s="23"/>
+      <c r="C51" s="33"/>
+      <c r="D51" s="12"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="33"/>
+      <c r="J51" s="32"/>
+    </row>
+    <row r="52" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B52" s="23"/>
+      <c r="C52" s="33"/>
+      <c r="D52" s="12"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="33"/>
+      <c r="J52" s="32"/>
+    </row>
+    <row r="53" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B53" s="23"/>
+      <c r="C53" s="33"/>
+      <c r="D53" s="12"/>
+      <c r="E53" s="3"/>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
+      <c r="H53" s="3"/>
+      <c r="I53" s="33"/>
+      <c r="J53" s="32"/>
+    </row>
+    <row r="54" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B54" s="23"/>
+      <c r="C54" s="33"/>
+      <c r="D54" s="12"/>
+      <c r="E54" s="3"/>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
+      <c r="I54" s="33"/>
+      <c r="J54" s="32"/>
+    </row>
+    <row r="55" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B55" s="23"/>
+      <c r="C55" s="33"/>
+      <c r="D55" s="12"/>
+      <c r="E55" s="3"/>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+      <c r="H55" s="3"/>
+      <c r="I55" s="33"/>
+      <c r="J55" s="32"/>
+    </row>
+    <row r="56" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B56" s="23"/>
+      <c r="C56" s="33"/>
+      <c r="D56" s="12"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
+      <c r="H56" s="3"/>
+      <c r="I56" s="33"/>
+      <c r="J56" s="32"/>
+    </row>
+    <row r="57" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B57" s="23"/>
+      <c r="C57" s="33"/>
+      <c r="D57" s="12"/>
+      <c r="E57" s="3"/>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="3"/>
+      <c r="I57" s="33"/>
+      <c r="J57" s="32"/>
+    </row>
+    <row r="58" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B58" s="23"/>
+      <c r="C58" s="33"/>
+      <c r="D58" s="12"/>
+      <c r="E58" s="3"/>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
+      <c r="H58" s="3"/>
+      <c r="I58" s="33"/>
+      <c r="J58" s="32"/>
+    </row>
+    <row r="59" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B59" s="23"/>
+      <c r="C59" s="33"/>
+      <c r="D59" s="12"/>
+      <c r="E59" s="3"/>
+      <c r="F59" s="3"/>
+      <c r="G59" s="3"/>
+      <c r="H59" s="3"/>
+      <c r="I59" s="33"/>
+      <c r="J59" s="32"/>
+    </row>
+    <row r="60" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B60" s="23"/>
+      <c r="C60" s="33"/>
+      <c r="D60" s="12"/>
+      <c r="E60" s="3"/>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
+      <c r="I60" s="33"/>
+      <c r="J60" s="32"/>
+    </row>
+    <row r="61" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B61" s="23"/>
+      <c r="C61" s="33"/>
+      <c r="D61" s="12"/>
+      <c r="E61" s="3"/>
+      <c r="F61" s="3"/>
+      <c r="G61" s="3"/>
+      <c r="H61" s="3"/>
+      <c r="I61" s="33"/>
+      <c r="J61" s="32"/>
+    </row>
+    <row r="62" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B62" s="23"/>
+      <c r="C62" s="33"/>
+      <c r="D62" s="12"/>
+      <c r="E62" s="3"/>
+      <c r="F62" s="3"/>
+      <c r="G62" s="3"/>
+      <c r="H62" s="3"/>
+      <c r="I62" s="33"/>
+      <c r="J62" s="32"/>
+    </row>
+    <row r="63" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B63" s="23"/>
+      <c r="C63" s="33"/>
+      <c r="D63" s="12"/>
+      <c r="E63" s="3"/>
+      <c r="F63" s="3"/>
+      <c r="G63" s="3"/>
+      <c r="H63" s="3"/>
+      <c r="I63" s="33"/>
+      <c r="J63" s="32"/>
+    </row>
+    <row r="64" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B64" s="24"/>
+      <c r="C64" s="36"/>
+      <c r="D64" s="13"/>
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+      <c r="G64" s="5"/>
+      <c r="H64" s="5"/>
+      <c r="I64" s="36"/>
+      <c r="J64" s="32"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="2">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3E12C11-8B88-45B7-BD25-4E819046FF08}">
   <dimension ref="B2:I32"/>
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1563,7 +2859,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2FA5E18-19A2-4DA7-9A95-328DE2FBBD0C}">
   <dimension ref="B2:G32"/>
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1876,7 +3172,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6DC10A0-2F8B-491B-B923-1486860B0A91}">
   <dimension ref="B2:G32"/>
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2189,7 +3485,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{014593E6-C137-4A83-B335-8EC85FCC951C}">
   <dimension ref="B2:G32"/>
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2502,7 +3798,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B872F986-AA11-4310-9F15-06BC0BD7DCB4}">
   <dimension ref="B4:G33"/>
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>